<commit_message>
Final Update on Schematics
</commit_message>
<xml_diff>
--- a/G-Alert-BOM.xlsx
+++ b/G-Alert-BOM.xlsx
@@ -1,30 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saikat.c\Desktop\G-Alert\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/174a02a4545e672e/Desktop/G-Alert/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_7267A3ADC5CE458BCDA7AEE91DD2A52570F6C279" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{C47D176F-1C93-4CCD-AE23-E0B46E35C73C}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="G-Alert-BOM" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Saikat Chakraborty(1025235)</author>
   </authors>
   <commentList>
-    <comment ref="A6" authorId="0" shapeId="0">
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -193,7 +204,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -705,7 +716,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -752,6 +763,7 @@
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="42" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="42" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1107,21 +1119,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="5"/>
-    <col min="3" max="3" width="16.85546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" style="5" customWidth="1"/>
+    <col min="1" max="1" width="27.5546875" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="5"/>
+    <col min="3" max="3" width="16.88671875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="5" customWidth="1"/>
     <col min="5" max="5" width="21" style="5" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" style="9" customWidth="1"/>
-    <col min="7" max="7" width="67.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="9" customWidth="1"/>
+    <col min="7" max="7" width="67.109375" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1144,12 +1156,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
@@ -1164,12 +1176,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>29</v>
       </c>
       <c r="B3" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>6</v>
@@ -1184,12 +1196,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>26</v>
       </c>
       <c r="B4" s="15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>37</v>
@@ -1204,12 +1216,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>39</v>
@@ -1224,12 +1236,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>27</v>
       </c>
       <c r="B6" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>21</v>
@@ -1238,21 +1250,21 @@
         <v>43</v>
       </c>
       <c r="E6" s="11">
-        <v>150</v>
+        <v>185</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="18" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>24</v>
@@ -1267,20 +1279,20 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>36</v>
       </c>
       <c r="B8" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>8</v>
@@ -1292,12 +1304,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>10</v>
@@ -1309,12 +1321,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="B12" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>12</v>
@@ -1326,12 +1338,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>14</v>
@@ -1346,12 +1358,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="5">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>16</v>
@@ -1364,15 +1376,15 @@
       </c>
       <c r="G14" s="7">
         <f>SUMPRODUCT(B:B,E:E)</f>
-        <v>436</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1093</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>18</v>
@@ -1384,12 +1396,12 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>20</v>
@@ -1401,7 +1413,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -1418,14 +1430,15 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="F3" r:id="rId2"/>
-    <hyperlink ref="F7" r:id="rId3"/>
-    <hyperlink ref="F5" r:id="rId4"/>
-    <hyperlink ref="F6" r:id="rId5"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="G6" r:id="rId6" xr:uid="{D3805FF2-9636-42CE-ACE2-27A17C6D98DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" r:id="rId6"/>
-  <legacyDrawing r:id="rId7"/>
+  <pageSetup orientation="landscape" r:id="rId7"/>
+  <legacyDrawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>